<commit_message>
move the imputation qc where it belongs, and make it show BH instead of only pi
</commit_message>
<xml_diff>
--- a/02_Normalization/imputation/c_data/imputation_qc_source_data.xlsx
+++ b/02_Normalization/imputation/c_data/imputation_qc_source_data.xlsx
@@ -7,14 +7,14 @@
   </bookViews>
   <sheets>
     <sheet name="overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="logfc_concordance" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="pi_counts" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="bh_vs_pi" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="logfc_concordance" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="21" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="31" uniqueCount="31">
   <si>
     <t xml:space="preserve">sheet</t>
   </si>
@@ -22,16 +22,16 @@
     <t xml:space="preserve">description</t>
   </si>
   <si>
+    <t xml:space="preserve">bh_vs_pi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Panels A-B: BH q&lt;0.10 and Pi&lt;0.05 protein counts per method per key contrast</t>
+  </si>
+  <si>
     <t xml:space="preserve">logfc_concordance</t>
   </si>
   <si>
-    <t xml:space="preserve">Panel A: Spearman rho of each imputed arm's per-protein logFC vs the non-imputed reference, key contrasts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">pi_counts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Panel B: pi-significant protein count per method per key contrast</t>
+    <t xml:space="preserve">Panel C: median Spearman rho of each imputed arm's per-protein logFC vs the non-imputed reference, split by per-protein missingness</t>
   </si>
   <si>
     <t xml:space="preserve">contrast</t>
@@ -40,43 +40,73 @@
     <t xml:space="preserve">method</t>
   </si>
   <si>
+    <t xml:space="preserve">n_BH_10</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n_BH_05</t>
+  </si>
+  <si>
+    <t xml:space="preserve">n_pi</t>
+  </si>
+  <si>
+    <t xml:space="preserve">is_null_contrast</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acute_HR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">imp4p</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acute_HRvLR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acute_Interaction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Acute_LR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Baseline_HRvLR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trained_HRvLR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Training_HR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Training_Interaction</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Training_LR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">missForest</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MsCoreUtils</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Non-imputed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Perseus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">stratum</t>
+  </si>
+  <si>
     <t xml:space="preserve">rho</t>
   </si>
   <si>
-    <t xml:space="preserve">n</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Acute_HR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">missForest</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Acute_LR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Baseline_HRvLR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Training_HR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Training_LR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">imp4p</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MsCoreUtils</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Perseus</t>
-  </si>
-  <si>
-    <t xml:space="preserve">n_pi</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Non-imputed</t>
+    <t xml:space="preserve">0 (imputation is a no-op)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1-9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">&gt;=10</t>
   </si>
 </sst>
 </file>
@@ -453,285 +483,911 @@
       <c r="D1" t="s">
         <v>9</v>
       </c>
+      <c r="E1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F1" t="s">
+        <v>11</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="B2" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C2" t="n">
-        <v>0.974769577227448</v>
+        <v>38</v>
       </c>
       <c r="D2" t="n">
-        <v>1896</v>
+        <v>26</v>
+      </c>
+      <c r="E2" t="n">
+        <v>135</v>
+      </c>
+      <c r="F2" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="B3" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C3" t="n">
-        <v>0.968419608745761</v>
+        <v>23</v>
       </c>
       <c r="D3" t="n">
-        <v>1896</v>
+        <v>19</v>
+      </c>
+      <c r="E3" t="n">
+        <v>97</v>
+      </c>
+      <c r="F3" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
+        <v>15</v>
+      </c>
+      <c r="B4" t="s">
         <v>13</v>
       </c>
-      <c r="B4" t="s">
-        <v>11</v>
-      </c>
       <c r="C4" t="n">
-        <v>0.950568005846472</v>
+        <v>25</v>
       </c>
       <c r="D4" t="n">
-        <v>1896</v>
+        <v>22</v>
+      </c>
+      <c r="E4" t="n">
+        <v>143</v>
+      </c>
+      <c r="F4" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="B5" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C5" t="n">
-        <v>0.96281300521173</v>
+        <v>63</v>
       </c>
       <c r="D5" t="n">
-        <v>1896</v>
+        <v>45</v>
+      </c>
+      <c r="E5" t="n">
+        <v>112</v>
+      </c>
+      <c r="F5" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="B6" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="C6" t="n">
-        <v>0.967849645743138</v>
+        <v>28</v>
       </c>
       <c r="D6" t="n">
-        <v>1896</v>
+        <v>27</v>
+      </c>
+      <c r="E6" t="n">
+        <v>88</v>
+      </c>
+      <c r="F6" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>10</v>
+        <v>18</v>
       </c>
       <c r="B7" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C7" t="n">
-        <v>0.935686097178357</v>
+        <v>8</v>
       </c>
       <c r="D7" t="n">
-        <v>1896</v>
+        <v>6</v>
+      </c>
+      <c r="E7" t="n">
+        <v>60</v>
+      </c>
+      <c r="F7" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="B8" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C8" t="n">
-        <v>0.931109135412394</v>
+        <v>53</v>
       </c>
       <c r="D8" t="n">
-        <v>1896</v>
+        <v>42</v>
+      </c>
+      <c r="E8" t="n">
+        <v>120</v>
+      </c>
+      <c r="F8" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
+        <v>20</v>
+      </c>
+      <c r="B9" t="s">
         <v>13</v>
       </c>
-      <c r="B9" t="s">
-        <v>16</v>
-      </c>
       <c r="C9" t="n">
-        <v>0.900074242178623</v>
+        <v>33</v>
       </c>
       <c r="D9" t="n">
-        <v>1896</v>
+        <v>27</v>
+      </c>
+      <c r="E9" t="n">
+        <v>115</v>
+      </c>
+      <c r="F9" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="B10" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C10" t="n">
-        <v>0.909546096622222</v>
+        <v>20</v>
       </c>
       <c r="D10" t="n">
-        <v>1896</v>
+        <v>18</v>
+      </c>
+      <c r="E10" t="n">
+        <v>64</v>
+      </c>
+      <c r="F10" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="B11" t="s">
-        <v>16</v>
+        <v>22</v>
       </c>
       <c r="C11" t="n">
-        <v>0.903690871641575</v>
+        <v>2</v>
       </c>
       <c r="D11" t="n">
-        <v>1896</v>
+        <v>0</v>
+      </c>
+      <c r="E11" t="n">
+        <v>59</v>
+      </c>
+      <c r="F11" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>10</v>
+        <v>14</v>
       </c>
       <c r="B12" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="C12" t="n">
-        <v>0.867298901495622</v>
+        <v>0</v>
       </c>
       <c r="D12" t="n">
-        <v>1896</v>
+        <v>0</v>
+      </c>
+      <c r="E12" t="n">
+        <v>42</v>
+      </c>
+      <c r="F12" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="B13" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="C13" t="n">
-        <v>0.870330543090063</v>
+        <v>0</v>
       </c>
       <c r="D13" t="n">
-        <v>1896</v>
+        <v>0</v>
+      </c>
+      <c r="E13" t="n">
+        <v>67</v>
+      </c>
+      <c r="F13" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="s">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="B14" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="C14" t="n">
-        <v>0.841956063260182</v>
+        <v>30</v>
       </c>
       <c r="D14" t="n">
-        <v>1896</v>
+        <v>20</v>
+      </c>
+      <c r="E14" t="n">
+        <v>64</v>
+      </c>
+      <c r="F14" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="s">
-        <v>14</v>
+        <v>17</v>
       </c>
       <c r="B15" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="C15" t="n">
-        <v>0.859214382202245</v>
+        <v>0</v>
       </c>
       <c r="D15" t="n">
-        <v>1896</v>
+        <v>0</v>
+      </c>
+      <c r="E15" t="n">
+        <v>8</v>
+      </c>
+      <c r="F15" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="s">
-        <v>15</v>
+        <v>18</v>
       </c>
       <c r="B16" t="s">
-        <v>17</v>
+        <v>22</v>
       </c>
       <c r="C16" t="n">
-        <v>0.850066347765401</v>
+        <v>0</v>
       </c>
       <c r="D16" t="n">
-        <v>1896</v>
+        <v>0</v>
+      </c>
+      <c r="E16" t="n">
+        <v>12</v>
+      </c>
+      <c r="F16" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="s">
-        <v>10</v>
+        <v>19</v>
       </c>
       <c r="B17" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C17" t="n">
-        <v>0.574440558337026</v>
+        <v>0</v>
       </c>
       <c r="D17" t="n">
-        <v>1896</v>
+        <v>0</v>
+      </c>
+      <c r="E17" t="n">
+        <v>25</v>
+      </c>
+      <c r="F17" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="s">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="B18" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C18" t="n">
-        <v>0.531309933231697</v>
+        <v>0</v>
       </c>
       <c r="D18" t="n">
-        <v>1896</v>
+        <v>0</v>
+      </c>
+      <c r="E18" t="n">
+        <v>15</v>
+      </c>
+      <c r="F18" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="s">
-        <v>13</v>
+        <v>21</v>
       </c>
       <c r="B19" t="s">
-        <v>18</v>
+        <v>22</v>
       </c>
       <c r="C19" t="n">
-        <v>0.358504687202276</v>
+        <v>0</v>
       </c>
       <c r="D19" t="n">
-        <v>1896</v>
+        <v>0</v>
+      </c>
+      <c r="E19" t="n">
+        <v>12</v>
+      </c>
+      <c r="F19" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="B20" t="s">
-        <v>18</v>
+        <v>23</v>
       </c>
       <c r="C20" t="n">
-        <v>0.446372015636742</v>
+        <v>2</v>
       </c>
       <c r="D20" t="n">
-        <v>1896</v>
+        <v>0</v>
+      </c>
+      <c r="E20" t="n">
+        <v>80</v>
+      </c>
+      <c r="F20" t="b">
+        <v>0</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="s">
+        <v>14</v>
+      </c>
+      <c r="B21" t="s">
+        <v>23</v>
+      </c>
+      <c r="C21" t="n">
+        <v>0</v>
+      </c>
+      <c r="D21" t="n">
+        <v>0</v>
+      </c>
+      <c r="E21" t="n">
+        <v>64</v>
+      </c>
+      <c r="F21" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="s">
         <v>15</v>
       </c>
-      <c r="B21" t="s">
+      <c r="B22" t="s">
+        <v>23</v>
+      </c>
+      <c r="C22" t="n">
+        <v>0</v>
+      </c>
+      <c r="D22" t="n">
+        <v>0</v>
+      </c>
+      <c r="E22" t="n">
+        <v>100</v>
+      </c>
+      <c r="F22" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="s">
+        <v>16</v>
+      </c>
+      <c r="B23" t="s">
+        <v>23</v>
+      </c>
+      <c r="C23" t="n">
+        <v>32</v>
+      </c>
+      <c r="D23" t="n">
+        <v>22</v>
+      </c>
+      <c r="E23" t="n">
+        <v>107</v>
+      </c>
+      <c r="F23" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="s">
+        <v>17</v>
+      </c>
+      <c r="B24" t="s">
+        <v>23</v>
+      </c>
+      <c r="C24" t="n">
+        <v>0</v>
+      </c>
+      <c r="D24" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" t="n">
+        <v>30</v>
+      </c>
+      <c r="F24" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="s">
         <v>18</v>
       </c>
-      <c r="C21" t="n">
-        <v>0.453801549348829</v>
-      </c>
-      <c r="D21" t="n">
-        <v>1896</v>
+      <c r="B25" t="s">
+        <v>23</v>
+      </c>
+      <c r="C25" t="n">
+        <v>0</v>
+      </c>
+      <c r="D25" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" t="n">
+        <v>36</v>
+      </c>
+      <c r="F25" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="s">
+        <v>19</v>
+      </c>
+      <c r="B26" t="s">
+        <v>23</v>
+      </c>
+      <c r="C26" t="n">
+        <v>0</v>
+      </c>
+      <c r="D26" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" t="n">
+        <v>49</v>
+      </c>
+      <c r="F26" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="s">
+        <v>20</v>
+      </c>
+      <c r="B27" t="s">
+        <v>23</v>
+      </c>
+      <c r="C27" t="n">
+        <v>0</v>
+      </c>
+      <c r="D27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" t="n">
+        <v>39</v>
+      </c>
+      <c r="F27" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="s">
+        <v>21</v>
+      </c>
+      <c r="B28" t="s">
+        <v>23</v>
+      </c>
+      <c r="C28" t="n">
+        <v>3</v>
+      </c>
+      <c r="D28" t="n">
+        <v>0</v>
+      </c>
+      <c r="E28" t="n">
+        <v>49</v>
+      </c>
+      <c r="F28" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="s">
+        <v>12</v>
+      </c>
+      <c r="B29" t="s">
+        <v>24</v>
+      </c>
+      <c r="C29" t="n">
+        <v>2</v>
+      </c>
+      <c r="D29" t="n">
+        <v>0</v>
+      </c>
+      <c r="E29" t="n">
+        <v>84</v>
+      </c>
+      <c r="F29" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="s">
+        <v>14</v>
+      </c>
+      <c r="B30" t="s">
+        <v>24</v>
+      </c>
+      <c r="C30" t="n">
+        <v>0</v>
+      </c>
+      <c r="D30" t="n">
+        <v>0</v>
+      </c>
+      <c r="E30" t="n">
+        <v>51</v>
+      </c>
+      <c r="F30" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="s">
+        <v>15</v>
+      </c>
+      <c r="B31" t="s">
+        <v>24</v>
+      </c>
+      <c r="C31" t="n">
+        <v>0</v>
+      </c>
+      <c r="D31" t="n">
+        <v>0</v>
+      </c>
+      <c r="E31" t="n">
+        <v>91</v>
+      </c>
+      <c r="F31" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="s">
+        <v>16</v>
+      </c>
+      <c r="B32" t="s">
+        <v>24</v>
+      </c>
+      <c r="C32" t="n">
+        <v>19</v>
+      </c>
+      <c r="D32" t="n">
+        <v>15</v>
+      </c>
+      <c r="E32" t="n">
+        <v>81</v>
+      </c>
+      <c r="F32" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="s">
+        <v>17</v>
+      </c>
+      <c r="B33" t="s">
+        <v>24</v>
+      </c>
+      <c r="C33" t="n">
+        <v>0</v>
+      </c>
+      <c r="D33" t="n">
+        <v>0</v>
+      </c>
+      <c r="E33" t="n">
+        <v>30</v>
+      </c>
+      <c r="F33" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="s">
+        <v>18</v>
+      </c>
+      <c r="B34" t="s">
+        <v>24</v>
+      </c>
+      <c r="C34" t="n">
+        <v>0</v>
+      </c>
+      <c r="D34" t="n">
+        <v>0</v>
+      </c>
+      <c r="E34" t="n">
+        <v>33</v>
+      </c>
+      <c r="F34" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="s">
+        <v>19</v>
+      </c>
+      <c r="B35" t="s">
+        <v>24</v>
+      </c>
+      <c r="C35" t="n">
+        <v>0</v>
+      </c>
+      <c r="D35" t="n">
+        <v>0</v>
+      </c>
+      <c r="E35" t="n">
+        <v>54</v>
+      </c>
+      <c r="F35" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="s">
+        <v>20</v>
+      </c>
+      <c r="B36" t="s">
+        <v>24</v>
+      </c>
+      <c r="C36" t="n">
+        <v>0</v>
+      </c>
+      <c r="D36" t="n">
+        <v>0</v>
+      </c>
+      <c r="E36" t="n">
+        <v>56</v>
+      </c>
+      <c r="F36" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="s">
+        <v>21</v>
+      </c>
+      <c r="B37" t="s">
+        <v>24</v>
+      </c>
+      <c r="C37" t="n">
+        <v>0</v>
+      </c>
+      <c r="D37" t="n">
+        <v>0</v>
+      </c>
+      <c r="E37" t="n">
+        <v>26</v>
+      </c>
+      <c r="F37" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="s">
+        <v>12</v>
+      </c>
+      <c r="B38" t="s">
+        <v>25</v>
+      </c>
+      <c r="C38" t="n">
+        <v>0</v>
+      </c>
+      <c r="D38" t="n">
+        <v>0</v>
+      </c>
+      <c r="E38" t="n">
+        <v>196</v>
+      </c>
+      <c r="F38" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="s">
+        <v>14</v>
+      </c>
+      <c r="B39" t="s">
+        <v>25</v>
+      </c>
+      <c r="C39" t="n">
+        <v>0</v>
+      </c>
+      <c r="D39" t="n">
+        <v>0</v>
+      </c>
+      <c r="E39" t="n">
+        <v>197</v>
+      </c>
+      <c r="F39" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="s">
+        <v>15</v>
+      </c>
+      <c r="B40" t="s">
+        <v>25</v>
+      </c>
+      <c r="C40" t="n">
+        <v>0</v>
+      </c>
+      <c r="D40" t="n">
+        <v>0</v>
+      </c>
+      <c r="E40" t="n">
+        <v>233</v>
+      </c>
+      <c r="F40" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="s">
+        <v>16</v>
+      </c>
+      <c r="B41" t="s">
+        <v>25</v>
+      </c>
+      <c r="C41" t="n">
+        <v>21</v>
+      </c>
+      <c r="D41" t="n">
+        <v>16</v>
+      </c>
+      <c r="E41" t="n">
+        <v>222</v>
+      </c>
+      <c r="F41" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="s">
+        <v>17</v>
+      </c>
+      <c r="B42" t="s">
+        <v>25</v>
+      </c>
+      <c r="C42" t="n">
+        <v>0</v>
+      </c>
+      <c r="D42" t="n">
+        <v>0</v>
+      </c>
+      <c r="E42" t="n">
+        <v>139</v>
+      </c>
+      <c r="F42" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="s">
+        <v>18</v>
+      </c>
+      <c r="B43" t="s">
+        <v>25</v>
+      </c>
+      <c r="C43" t="n">
+        <v>0</v>
+      </c>
+      <c r="D43" t="n">
+        <v>0</v>
+      </c>
+      <c r="E43" t="n">
+        <v>94</v>
+      </c>
+      <c r="F43" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="s">
+        <v>19</v>
+      </c>
+      <c r="B44" t="s">
+        <v>25</v>
+      </c>
+      <c r="C44" t="n">
+        <v>0</v>
+      </c>
+      <c r="D44" t="n">
+        <v>0</v>
+      </c>
+      <c r="E44" t="n">
+        <v>185</v>
+      </c>
+      <c r="F44" t="b">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="s">
+        <v>20</v>
+      </c>
+      <c r="B45" t="s">
+        <v>25</v>
+      </c>
+      <c r="C45" t="n">
+        <v>0</v>
+      </c>
+      <c r="D45" t="n">
+        <v>0</v>
+      </c>
+      <c r="E45" t="n">
+        <v>148</v>
+      </c>
+      <c r="F45" t="b">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="s">
+        <v>21</v>
+      </c>
+      <c r="B46" t="s">
+        <v>25</v>
+      </c>
+      <c r="C46" t="n">
+        <v>0</v>
+      </c>
+      <c r="D46" t="n">
+        <v>0</v>
+      </c>
+      <c r="E46" t="n">
+        <v>118</v>
+      </c>
+      <c r="F46" t="b">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -747,288 +1403,145 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B1" t="s">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="C1" t="s">
-        <v>7</v>
+        <v>27</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>14</v>
-      </c>
-      <c r="B2" t="n">
-        <v>54</v>
-      </c>
-      <c r="C2" t="s">
-        <v>20</v>
+        <v>22</v>
+      </c>
+      <c r="B2" t="s">
+        <v>28</v>
+      </c>
+      <c r="C2" t="n">
+        <v>0.999988046095852</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>15</v>
-      </c>
-      <c r="B3" t="n">
-        <v>25</v>
-      </c>
-      <c r="C3" t="s">
-        <v>20</v>
+        <v>22</v>
+      </c>
+      <c r="B3" t="s">
+        <v>29</v>
+      </c>
+      <c r="C3" t="n">
+        <v>0.984672248455361</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>10</v>
-      </c>
-      <c r="B4" t="n">
-        <v>84</v>
-      </c>
-      <c r="C4" t="s">
-        <v>20</v>
+        <v>22</v>
+      </c>
+      <c r="B4" t="s">
+        <v>30</v>
+      </c>
+      <c r="C4" t="n">
+        <v>0.919979603820525</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>12</v>
-      </c>
-      <c r="B5" t="n">
-        <v>76</v>
-      </c>
-      <c r="C5" t="s">
-        <v>20</v>
+        <v>13</v>
+      </c>
+      <c r="B5" t="s">
+        <v>28</v>
+      </c>
+      <c r="C5" t="n">
+        <v>0.999937135017208</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
         <v>13</v>
       </c>
-      <c r="B6" t="n">
-        <v>28</v>
-      </c>
-      <c r="C6" t="s">
-        <v>20</v>
+      <c r="B6" t="s">
+        <v>29</v>
+      </c>
+      <c r="C6" t="n">
+        <v>0.932169215576077</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>10</v>
-      </c>
-      <c r="B7" t="n">
-        <v>57</v>
-      </c>
-      <c r="C7" t="s">
-        <v>11</v>
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
+        <v>30</v>
+      </c>
+      <c r="C7" t="n">
+        <v>0.869921734270971</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="s">
-        <v>12</v>
-      </c>
-      <c r="B8" t="n">
-        <v>60</v>
-      </c>
-      <c r="C8" t="s">
-        <v>11</v>
+        <v>23</v>
+      </c>
+      <c r="B8" t="s">
+        <v>28</v>
+      </c>
+      <c r="C8" t="n">
+        <v>0.999974180708225</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="s">
-        <v>13</v>
-      </c>
-      <c r="B9" t="n">
-        <v>7</v>
-      </c>
-      <c r="C9" t="s">
-        <v>11</v>
+        <v>23</v>
+      </c>
+      <c r="B9" t="s">
+        <v>29</v>
+      </c>
+      <c r="C9" t="n">
+        <v>0.968866559259355</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="s">
-        <v>14</v>
-      </c>
-      <c r="B10" t="n">
         <v>23</v>
       </c>
-      <c r="C10" t="s">
-        <v>11</v>
+      <c r="B10" t="s">
+        <v>30</v>
+      </c>
+      <c r="C10" t="n">
+        <v>0.577834406847561</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="s">
-        <v>15</v>
-      </c>
-      <c r="B11" t="n">
-        <v>12</v>
-      </c>
-      <c r="C11" t="s">
-        <v>11</v>
+        <v>25</v>
+      </c>
+      <c r="B11" t="s">
+        <v>28</v>
+      </c>
+      <c r="C11" t="n">
+        <v>0.999946749493814</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="s">
-        <v>10</v>
-      </c>
-      <c r="B12" t="n">
-        <v>127</v>
-      </c>
-      <c r="C12" t="s">
-        <v>16</v>
+        <v>25</v>
+      </c>
+      <c r="B12" t="s">
+        <v>29</v>
+      </c>
+      <c r="C12" t="n">
+        <v>0.361536379302119</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="s">
-        <v>12</v>
-      </c>
-      <c r="B13" t="n">
-        <v>118</v>
-      </c>
-      <c r="C13" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" t="s">
-        <v>13</v>
-      </c>
-      <c r="B14" t="n">
-        <v>91</v>
-      </c>
-      <c r="C14" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="s">
-        <v>14</v>
-      </c>
-      <c r="B15" t="n">
-        <v>115</v>
-      </c>
-      <c r="C15" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="s">
-        <v>15</v>
-      </c>
-      <c r="B16" t="n">
-        <v>60</v>
-      </c>
-      <c r="C16" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" t="s">
-        <v>10</v>
-      </c>
-      <c r="B17" t="n">
-        <v>80</v>
-      </c>
-      <c r="C17" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" t="s">
-        <v>12</v>
-      </c>
-      <c r="B18" t="n">
-        <v>103</v>
-      </c>
-      <c r="C18" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" t="s">
-        <v>13</v>
-      </c>
-      <c r="B19" t="n">
-        <v>29</v>
-      </c>
-      <c r="C19" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" t="s">
-        <v>14</v>
-      </c>
-      <c r="B20" t="n">
-        <v>50</v>
-      </c>
-      <c r="C20" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" t="s">
-        <v>15</v>
-      </c>
-      <c r="B21" t="n">
-        <v>45</v>
-      </c>
-      <c r="C21" t="s">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="A22" t="s">
-        <v>10</v>
-      </c>
-      <c r="B22" t="n">
-        <v>205</v>
-      </c>
-      <c r="C22" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" t="s">
-        <v>12</v>
-      </c>
-      <c r="B23" t="n">
-        <v>223</v>
-      </c>
-      <c r="C23" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" t="s">
-        <v>13</v>
-      </c>
-      <c r="B24" t="n">
-        <v>122</v>
-      </c>
-      <c r="C24" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="A25" t="s">
-        <v>14</v>
-      </c>
-      <c r="B25" t="n">
-        <v>175</v>
-      </c>
-      <c r="C25" t="s">
-        <v>18</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="A26" t="s">
-        <v>15</v>
-      </c>
-      <c r="B26" t="n">
-        <v>102</v>
-      </c>
-      <c r="C26" t="s">
-        <v>18</v>
+        <v>25</v>
+      </c>
+      <c r="B13" t="s">
+        <v>30</v>
+      </c>
+      <c r="C13" t="n">
+        <v>0.191469489414695</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
confirm blood_cor removals against the red-cell proteome before dropping them
</commit_message>
<xml_diff>
--- a/02_Normalization/imputation/c_data/imputation_qc_source_data.xlsx
+++ b/02_Normalization/imputation/c_data/imputation_qc_source_data.xlsx
@@ -498,13 +498,13 @@
         <v>13</v>
       </c>
       <c r="C2" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="D2" t="n">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="E2" t="n">
-        <v>135</v>
+        <v>126</v>
       </c>
       <c r="F2" t="b">
         <v>0</v>
@@ -521,10 +521,10 @@
         <v>23</v>
       </c>
       <c r="D3" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E3" t="n">
-        <v>97</v>
+        <v>82</v>
       </c>
       <c r="F3" t="b">
         <v>1</v>
@@ -538,13 +538,13 @@
         <v>13</v>
       </c>
       <c r="C4" t="n">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D4" t="n">
-        <v>22</v>
+        <v>20</v>
       </c>
       <c r="E4" t="n">
-        <v>143</v>
+        <v>136</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>
@@ -558,13 +558,13 @@
         <v>13</v>
       </c>
       <c r="C5" t="n">
-        <v>63</v>
+        <v>47</v>
       </c>
       <c r="D5" t="n">
-        <v>45</v>
+        <v>36</v>
       </c>
       <c r="E5" t="n">
-        <v>112</v>
+        <v>103</v>
       </c>
       <c r="F5" t="b">
         <v>0</v>
@@ -578,13 +578,13 @@
         <v>13</v>
       </c>
       <c r="C6" t="n">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D6" t="n">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="E6" t="n">
-        <v>88</v>
+        <v>91</v>
       </c>
       <c r="F6" t="b">
         <v>1</v>
@@ -598,13 +598,13 @@
         <v>13</v>
       </c>
       <c r="C7" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="D7" t="n">
         <v>6</v>
       </c>
       <c r="E7" t="n">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="F7" t="b">
         <v>1</v>
@@ -618,13 +618,13 @@
         <v>13</v>
       </c>
       <c r="C8" t="n">
-        <v>53</v>
+        <v>47</v>
       </c>
       <c r="D8" t="n">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="E8" t="n">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="F8" t="b">
         <v>0</v>
@@ -638,13 +638,13 @@
         <v>13</v>
       </c>
       <c r="C9" t="n">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="D9" t="n">
         <v>27</v>
       </c>
       <c r="E9" t="n">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="F9" t="b">
         <v>1</v>
@@ -664,7 +664,7 @@
         <v>18</v>
       </c>
       <c r="E10" t="n">
-        <v>64</v>
+        <v>55</v>
       </c>
       <c r="F10" t="b">
         <v>0</v>
@@ -704,7 +704,7 @@
         <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>42</v>
+        <v>29</v>
       </c>
       <c r="F12" t="b">
         <v>1</v>
@@ -724,7 +724,7 @@
         <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>67</v>
+        <v>48</v>
       </c>
       <c r="F13" t="b">
         <v>1</v>
@@ -738,13 +738,13 @@
         <v>22</v>
       </c>
       <c r="C14" t="n">
-        <v>30</v>
+        <v>11</v>
       </c>
       <c r="D14" t="n">
-        <v>20</v>
+        <v>9</v>
       </c>
       <c r="E14" t="n">
-        <v>64</v>
+        <v>52</v>
       </c>
       <c r="F14" t="b">
         <v>0</v>
@@ -784,7 +784,7 @@
         <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F16" t="b">
         <v>1</v>
@@ -804,7 +804,7 @@
         <v>0</v>
       </c>
       <c r="E17" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F17" t="b">
         <v>0</v>
@@ -824,7 +824,7 @@
         <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="F18" t="b">
         <v>1</v>
@@ -844,7 +844,7 @@
         <v>0</v>
       </c>
       <c r="E19" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F19" t="b">
         <v>0</v>
@@ -864,7 +864,7 @@
         <v>0</v>
       </c>
       <c r="E20" t="n">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="F20" t="b">
         <v>0</v>
@@ -884,7 +884,7 @@
         <v>0</v>
       </c>
       <c r="E21" t="n">
-        <v>64</v>
+        <v>52</v>
       </c>
       <c r="F21" t="b">
         <v>1</v>
@@ -904,7 +904,7 @@
         <v>0</v>
       </c>
       <c r="E22" t="n">
-        <v>100</v>
+        <v>91</v>
       </c>
       <c r="F22" t="b">
         <v>1</v>
@@ -918,13 +918,13 @@
         <v>23</v>
       </c>
       <c r="C23" t="n">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="D23" t="n">
-        <v>22</v>
+        <v>10</v>
       </c>
       <c r="E23" t="n">
-        <v>107</v>
+        <v>92</v>
       </c>
       <c r="F23" t="b">
         <v>0</v>
@@ -964,7 +964,7 @@
         <v>0</v>
       </c>
       <c r="E25" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F25" t="b">
         <v>1</v>
@@ -984,7 +984,7 @@
         <v>0</v>
       </c>
       <c r="E26" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F26" t="b">
         <v>0</v>
@@ -1004,7 +1004,7 @@
         <v>0</v>
       </c>
       <c r="E27" t="n">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="F27" t="b">
         <v>1</v>
@@ -1024,7 +1024,7 @@
         <v>0</v>
       </c>
       <c r="E28" t="n">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="F28" t="b">
         <v>0</v>
@@ -1044,7 +1044,7 @@
         <v>0</v>
       </c>
       <c r="E29" t="n">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="F29" t="b">
         <v>0</v>
@@ -1064,7 +1064,7 @@
         <v>0</v>
       </c>
       <c r="E30" t="n">
-        <v>51</v>
+        <v>44</v>
       </c>
       <c r="F30" t="b">
         <v>1</v>
@@ -1084,7 +1084,7 @@
         <v>0</v>
       </c>
       <c r="E31" t="n">
-        <v>91</v>
+        <v>79</v>
       </c>
       <c r="F31" t="b">
         <v>1</v>
@@ -1098,13 +1098,13 @@
         <v>24</v>
       </c>
       <c r="C32" t="n">
-        <v>19</v>
+        <v>9</v>
       </c>
       <c r="D32" t="n">
-        <v>15</v>
+        <v>8</v>
       </c>
       <c r="E32" t="n">
-        <v>81</v>
+        <v>69</v>
       </c>
       <c r="F32" t="b">
         <v>0</v>
@@ -1164,7 +1164,7 @@
         <v>0</v>
       </c>
       <c r="E35" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F35" t="b">
         <v>0</v>
@@ -1204,7 +1204,7 @@
         <v>0</v>
       </c>
       <c r="E37" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="F37" t="b">
         <v>0</v>
@@ -1224,7 +1224,7 @@
         <v>0</v>
       </c>
       <c r="E38" t="n">
-        <v>196</v>
+        <v>189</v>
       </c>
       <c r="F38" t="b">
         <v>0</v>
@@ -1244,7 +1244,7 @@
         <v>0</v>
       </c>
       <c r="E39" t="n">
-        <v>197</v>
+        <v>189</v>
       </c>
       <c r="F39" t="b">
         <v>1</v>
@@ -1264,7 +1264,7 @@
         <v>0</v>
       </c>
       <c r="E40" t="n">
-        <v>233</v>
+        <v>218</v>
       </c>
       <c r="F40" t="b">
         <v>1</v>
@@ -1278,13 +1278,13 @@
         <v>25</v>
       </c>
       <c r="C41" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="D41" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="E41" t="n">
-        <v>222</v>
+        <v>199</v>
       </c>
       <c r="F41" t="b">
         <v>0</v>
@@ -1304,7 +1304,7 @@
         <v>0</v>
       </c>
       <c r="E42" t="n">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="F42" t="b">
         <v>1</v>
@@ -1324,7 +1324,7 @@
         <v>0</v>
       </c>
       <c r="E43" t="n">
-        <v>94</v>
+        <v>85</v>
       </c>
       <c r="F43" t="b">
         <v>1</v>
@@ -1344,7 +1344,7 @@
         <v>0</v>
       </c>
       <c r="E44" t="n">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="F44" t="b">
         <v>0</v>
@@ -1364,7 +1364,7 @@
         <v>0</v>
       </c>
       <c r="E45" t="n">
-        <v>148</v>
+        <v>140</v>
       </c>
       <c r="F45" t="b">
         <v>1</v>
@@ -1384,7 +1384,7 @@
         <v>0</v>
       </c>
       <c r="E46" t="n">
-        <v>118</v>
+        <v>107</v>
       </c>
       <c r="F46" t="b">
         <v>0</v>
@@ -1420,7 +1420,7 @@
         <v>28</v>
       </c>
       <c r="C2" t="n">
-        <v>0.999988046095852</v>
+        <v>0.999988834485664</v>
       </c>
     </row>
     <row r="3">
@@ -1431,7 +1431,7 @@
         <v>29</v>
       </c>
       <c r="C3" t="n">
-        <v>0.984672248455361</v>
+        <v>0.985051312498553</v>
       </c>
     </row>
     <row r="4">
@@ -1442,7 +1442,7 @@
         <v>30</v>
       </c>
       <c r="C4" t="n">
-        <v>0.919979603820525</v>
+        <v>0.918075495861758</v>
       </c>
     </row>
     <row r="5">
@@ -1453,7 +1453,7 @@
         <v>28</v>
       </c>
       <c r="C5" t="n">
-        <v>0.999937135017208</v>
+        <v>0.999934967830002</v>
       </c>
     </row>
     <row r="6">
@@ -1464,7 +1464,7 @@
         <v>29</v>
       </c>
       <c r="C6" t="n">
-        <v>0.932169215576077</v>
+        <v>0.924449240608212</v>
       </c>
     </row>
     <row r="7">
@@ -1475,7 +1475,7 @@
         <v>30</v>
       </c>
       <c r="C7" t="n">
-        <v>0.869921734270971</v>
+        <v>0.869038454488801</v>
       </c>
     </row>
     <row r="8">
@@ -1486,7 +1486,7 @@
         <v>28</v>
       </c>
       <c r="C8" t="n">
-        <v>0.999974180708225</v>
+        <v>0.99997335202935</v>
       </c>
     </row>
     <row r="9">
@@ -1497,7 +1497,7 @@
         <v>29</v>
       </c>
       <c r="C9" t="n">
-        <v>0.968866559259355</v>
+        <v>0.968437496315169</v>
       </c>
     </row>
     <row r="10">
@@ -1508,7 +1508,7 @@
         <v>30</v>
       </c>
       <c r="C10" t="n">
-        <v>0.577834406847561</v>
+        <v>0.57619680269237</v>
       </c>
     </row>
     <row r="11">
@@ -1519,7 +1519,7 @@
         <v>28</v>
       </c>
       <c r="C11" t="n">
-        <v>0.999946749493814</v>
+        <v>0.999934894661494</v>
       </c>
     </row>
     <row r="12">
@@ -1530,7 +1530,7 @@
         <v>29</v>
       </c>
       <c r="C12" t="n">
-        <v>0.361536379302119</v>
+        <v>0.342050132915945</v>
       </c>
     </row>
     <row r="13">
@@ -1541,7 +1541,7 @@
         <v>30</v>
       </c>
       <c r="C13" t="n">
-        <v>0.191469489414695</v>
+        <v>0.218083280286436</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
regenerate every figure and workbook from the rebuilt pipeline
</commit_message>
<xml_diff>
--- a/02_Normalization/imputation/c_data/imputation_qc_source_data.xlsx
+++ b/02_Normalization/imputation/c_data/imputation_qc_source_data.xlsx
@@ -498,13 +498,13 @@
         <v>13</v>
       </c>
       <c r="C2" t="n">
-        <v>40</v>
+        <v>45</v>
       </c>
       <c r="D2" t="n">
-        <v>36</v>
+        <v>32</v>
       </c>
       <c r="E2" t="n">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="F2" t="b">
         <v>0</v>
@@ -518,13 +518,13 @@
         <v>13</v>
       </c>
       <c r="C3" t="n">
-        <v>23</v>
+        <v>28</v>
       </c>
       <c r="D3" t="n">
         <v>20</v>
       </c>
       <c r="E3" t="n">
-        <v>82</v>
+        <v>89</v>
       </c>
       <c r="F3" t="b">
         <v>1</v>
@@ -538,13 +538,13 @@
         <v>13</v>
       </c>
       <c r="C4" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="D4" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="E4" t="n">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>
@@ -558,13 +558,13 @@
         <v>13</v>
       </c>
       <c r="C5" t="n">
-        <v>47</v>
+        <v>41</v>
       </c>
       <c r="D5" t="n">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="E5" t="n">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="F5" t="b">
         <v>0</v>
@@ -578,13 +578,13 @@
         <v>13</v>
       </c>
       <c r="C6" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="D6" t="n">
-        <v>22</v>
+        <v>19</v>
       </c>
       <c r="E6" t="n">
-        <v>91</v>
+        <v>85</v>
       </c>
       <c r="F6" t="b">
         <v>1</v>
@@ -598,13 +598,13 @@
         <v>13</v>
       </c>
       <c r="C7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="D7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E7" t="n">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F7" t="b">
         <v>1</v>
@@ -618,13 +618,13 @@
         <v>13</v>
       </c>
       <c r="C8" t="n">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="D8" t="n">
-        <v>41</v>
+        <v>44</v>
       </c>
       <c r="E8" t="n">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="F8" t="b">
         <v>0</v>
@@ -638,13 +638,13 @@
         <v>13</v>
       </c>
       <c r="C9" t="n">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="D9" t="n">
-        <v>27</v>
+        <v>21</v>
       </c>
       <c r="E9" t="n">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="F9" t="b">
         <v>1</v>
@@ -658,13 +658,13 @@
         <v>13</v>
       </c>
       <c r="C10" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D10" t="n">
         <v>18</v>
       </c>
       <c r="E10" t="n">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="F10" t="b">
         <v>0</v>
@@ -704,7 +704,7 @@
         <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>29</v>
+        <v>34</v>
       </c>
       <c r="F12" t="b">
         <v>1</v>
@@ -724,7 +724,7 @@
         <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F13" t="b">
         <v>1</v>
@@ -738,13 +738,13 @@
         <v>22</v>
       </c>
       <c r="C14" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="D14" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="E14" t="n">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="F14" t="b">
         <v>0</v>
@@ -764,7 +764,7 @@
         <v>0</v>
       </c>
       <c r="E15" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F15" t="b">
         <v>1</v>
@@ -804,7 +804,7 @@
         <v>0</v>
       </c>
       <c r="E17" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F17" t="b">
         <v>0</v>
@@ -864,7 +864,7 @@
         <v>0</v>
       </c>
       <c r="E20" t="n">
-        <v>79</v>
+        <v>77</v>
       </c>
       <c r="F20" t="b">
         <v>0</v>
@@ -884,7 +884,7 @@
         <v>0</v>
       </c>
       <c r="E21" t="n">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="F21" t="b">
         <v>1</v>
@@ -904,7 +904,7 @@
         <v>0</v>
       </c>
       <c r="E22" t="n">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F22" t="b">
         <v>1</v>
@@ -918,13 +918,13 @@
         <v>23</v>
       </c>
       <c r="C23" t="n">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="D23" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="E23" t="n">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="F23" t="b">
         <v>0</v>
@@ -964,7 +964,7 @@
         <v>0</v>
       </c>
       <c r="E25" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F25" t="b">
         <v>1</v>
@@ -984,7 +984,7 @@
         <v>0</v>
       </c>
       <c r="E26" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="F26" t="b">
         <v>0</v>
@@ -1004,7 +1004,7 @@
         <v>0</v>
       </c>
       <c r="E27" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F27" t="b">
         <v>1</v>
@@ -1024,7 +1024,7 @@
         <v>0</v>
       </c>
       <c r="E28" t="n">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="F28" t="b">
         <v>0</v>
@@ -1044,7 +1044,7 @@
         <v>0</v>
       </c>
       <c r="E29" t="n">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="F29" t="b">
         <v>0</v>
@@ -1064,7 +1064,7 @@
         <v>0</v>
       </c>
       <c r="E30" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="F30" t="b">
         <v>1</v>
@@ -1084,7 +1084,7 @@
         <v>0</v>
       </c>
       <c r="E31" t="n">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="F31" t="b">
         <v>1</v>
@@ -1104,7 +1104,7 @@
         <v>8</v>
       </c>
       <c r="E32" t="n">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="F32" t="b">
         <v>0</v>
@@ -1224,7 +1224,7 @@
         <v>0</v>
       </c>
       <c r="E38" t="n">
-        <v>189</v>
+        <v>194</v>
       </c>
       <c r="F38" t="b">
         <v>0</v>
@@ -1244,7 +1244,7 @@
         <v>0</v>
       </c>
       <c r="E39" t="n">
-        <v>189</v>
+        <v>197</v>
       </c>
       <c r="F39" t="b">
         <v>1</v>
@@ -1264,7 +1264,7 @@
         <v>0</v>
       </c>
       <c r="E40" t="n">
-        <v>218</v>
+        <v>227</v>
       </c>
       <c r="F40" t="b">
         <v>1</v>
@@ -1278,13 +1278,13 @@
         <v>25</v>
       </c>
       <c r="C41" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="D41" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="E41" t="n">
-        <v>199</v>
+        <v>204</v>
       </c>
       <c r="F41" t="b">
         <v>0</v>
@@ -1304,7 +1304,7 @@
         <v>0</v>
       </c>
       <c r="E42" t="n">
-        <v>132</v>
+        <v>123</v>
       </c>
       <c r="F42" t="b">
         <v>1</v>
@@ -1324,7 +1324,7 @@
         <v>0</v>
       </c>
       <c r="E43" t="n">
-        <v>85</v>
+        <v>91</v>
       </c>
       <c r="F43" t="b">
         <v>1</v>
@@ -1338,13 +1338,13 @@
         <v>25</v>
       </c>
       <c r="C44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="D44" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="E44" t="n">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="F44" t="b">
         <v>0</v>
@@ -1364,7 +1364,7 @@
         <v>0</v>
       </c>
       <c r="E45" t="n">
-        <v>140</v>
+        <v>136</v>
       </c>
       <c r="F45" t="b">
         <v>1</v>
@@ -1384,7 +1384,7 @@
         <v>0</v>
       </c>
       <c r="E46" t="n">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="F46" t="b">
         <v>0</v>
@@ -1420,7 +1420,7 @@
         <v>28</v>
       </c>
       <c r="C2" t="n">
-        <v>0.999988834485664</v>
+        <v>0.99998789792876</v>
       </c>
     </row>
     <row r="3">
@@ -1431,7 +1431,7 @@
         <v>29</v>
       </c>
       <c r="C3" t="n">
-        <v>0.985051312498553</v>
+        <v>0.984982660004638</v>
       </c>
     </row>
     <row r="4">
@@ -1442,7 +1442,7 @@
         <v>30</v>
       </c>
       <c r="C4" t="n">
-        <v>0.918075495861758</v>
+        <v>0.919210023187344</v>
       </c>
     </row>
     <row r="5">
@@ -1453,7 +1453,7 @@
         <v>28</v>
       </c>
       <c r="C5" t="n">
-        <v>0.999934967830002</v>
+        <v>0.999931777683049</v>
       </c>
     </row>
     <row r="6">
@@ -1464,7 +1464,7 @@
         <v>29</v>
       </c>
       <c r="C6" t="n">
-        <v>0.924449240608212</v>
+        <v>0.939408933471279</v>
       </c>
     </row>
     <row r="7">
@@ -1475,7 +1475,7 @@
         <v>30</v>
       </c>
       <c r="C7" t="n">
-        <v>0.869038454488801</v>
+        <v>0.862872458707852</v>
       </c>
     </row>
     <row r="8">
@@ -1486,7 +1486,7 @@
         <v>28</v>
       </c>
       <c r="C8" t="n">
-        <v>0.99997335202935</v>
+        <v>0.999972913018302</v>
       </c>
     </row>
     <row r="9">
@@ -1497,7 +1497,7 @@
         <v>29</v>
       </c>
       <c r="C9" t="n">
-        <v>0.968437496315169</v>
+        <v>0.973581978807691</v>
       </c>
     </row>
     <row r="10">
@@ -1508,7 +1508,7 @@
         <v>30</v>
       </c>
       <c r="C10" t="n">
-        <v>0.57619680269237</v>
+        <v>0.577520510628317</v>
       </c>
     </row>
     <row r="11">
@@ -1519,7 +1519,7 @@
         <v>28</v>
       </c>
       <c r="C11" t="n">
-        <v>0.999934894661494</v>
+        <v>0.999935831218398</v>
       </c>
     </row>
     <row r="12">
@@ -1530,7 +1530,7 @@
         <v>29</v>
       </c>
       <c r="C12" t="n">
-        <v>0.342050132915945</v>
+        <v>0.343124640524274</v>
       </c>
     </row>
     <row r="13">
@@ -1541,7 +1541,7 @@
         <v>30</v>
       </c>
       <c r="C13" t="n">
-        <v>0.218083280286436</v>
+        <v>0.218701775211784</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
rerun normalization and DEP on the 1885-protein matrix
</commit_message>
<xml_diff>
--- a/02_Normalization/imputation/c_data/imputation_qc_source_data.xlsx
+++ b/02_Normalization/imputation/c_data/imputation_qc_source_data.xlsx
@@ -498,13 +498,13 @@
         <v>13</v>
       </c>
       <c r="C2" t="n">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="D2" t="n">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E2" t="n">
-        <v>129</v>
+        <v>117</v>
       </c>
       <c r="F2" t="b">
         <v>0</v>
@@ -518,13 +518,13 @@
         <v>13</v>
       </c>
       <c r="C3" t="n">
-        <v>28</v>
+        <v>20</v>
       </c>
       <c r="D3" t="n">
-        <v>20</v>
+        <v>16</v>
       </c>
       <c r="E3" t="n">
-        <v>89</v>
+        <v>77</v>
       </c>
       <c r="F3" t="b">
         <v>1</v>
@@ -541,10 +541,10 @@
         <v>25</v>
       </c>
       <c r="D4" t="n">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="E4" t="n">
-        <v>135</v>
+        <v>117</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>
@@ -558,13 +558,13 @@
         <v>13</v>
       </c>
       <c r="C5" t="n">
-        <v>41</v>
+        <v>38</v>
       </c>
       <c r="D5" t="n">
-        <v>33</v>
+        <v>27</v>
       </c>
       <c r="E5" t="n">
-        <v>102</v>
+        <v>90</v>
       </c>
       <c r="F5" t="b">
         <v>0</v>
@@ -578,13 +578,13 @@
         <v>13</v>
       </c>
       <c r="C6" t="n">
-        <v>28</v>
+        <v>25</v>
       </c>
       <c r="D6" t="n">
         <v>19</v>
       </c>
       <c r="E6" t="n">
-        <v>85</v>
+        <v>80</v>
       </c>
       <c r="F6" t="b">
         <v>1</v>
@@ -598,13 +598,13 @@
         <v>13</v>
       </c>
       <c r="C7" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="D7" t="n">
-        <v>7</v>
+        <v>4</v>
       </c>
       <c r="E7" t="n">
-        <v>64</v>
+        <v>57</v>
       </c>
       <c r="F7" t="b">
         <v>1</v>
@@ -618,13 +618,13 @@
         <v>13</v>
       </c>
       <c r="C8" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D8" t="n">
-        <v>44</v>
+        <v>38</v>
       </c>
       <c r="E8" t="n">
-        <v>111</v>
+        <v>119</v>
       </c>
       <c r="F8" t="b">
         <v>0</v>
@@ -638,13 +638,13 @@
         <v>13</v>
       </c>
       <c r="C9" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="D9" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E9" t="n">
-        <v>111</v>
+        <v>115</v>
       </c>
       <c r="F9" t="b">
         <v>1</v>
@@ -658,13 +658,13 @@
         <v>13</v>
       </c>
       <c r="C10" t="n">
+        <v>23</v>
+      </c>
+      <c r="D10" t="n">
         <v>21</v>
       </c>
-      <c r="D10" t="n">
-        <v>18</v>
-      </c>
       <c r="E10" t="n">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="F10" t="b">
         <v>0</v>
@@ -684,7 +684,7 @@
         <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="F11" t="b">
         <v>0</v>
@@ -704,7 +704,7 @@
         <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>34</v>
+        <v>26</v>
       </c>
       <c r="F12" t="b">
         <v>1</v>
@@ -724,7 +724,7 @@
         <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="F13" t="b">
         <v>1</v>
@@ -738,13 +738,13 @@
         <v>22</v>
       </c>
       <c r="C14" t="n">
-        <v>12</v>
+        <v>2</v>
       </c>
       <c r="D14" t="n">
-        <v>10</v>
+        <v>1</v>
       </c>
       <c r="E14" t="n">
-        <v>57</v>
+        <v>40</v>
       </c>
       <c r="F14" t="b">
         <v>0</v>
@@ -764,7 +764,7 @@
         <v>0</v>
       </c>
       <c r="E15" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F15" t="b">
         <v>1</v>
@@ -784,7 +784,7 @@
         <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F16" t="b">
         <v>1</v>
@@ -804,7 +804,7 @@
         <v>0</v>
       </c>
       <c r="E17" t="n">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F17" t="b">
         <v>0</v>
@@ -824,7 +824,7 @@
         <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F18" t="b">
         <v>1</v>
@@ -844,7 +844,7 @@
         <v>0</v>
       </c>
       <c r="E19" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F19" t="b">
         <v>0</v>
@@ -864,7 +864,7 @@
         <v>0</v>
       </c>
       <c r="E20" t="n">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="F20" t="b">
         <v>0</v>
@@ -884,7 +884,7 @@
         <v>0</v>
       </c>
       <c r="E21" t="n">
-        <v>55</v>
+        <v>49</v>
       </c>
       <c r="F21" t="b">
         <v>1</v>
@@ -904,7 +904,7 @@
         <v>0</v>
       </c>
       <c r="E22" t="n">
-        <v>93</v>
+        <v>86</v>
       </c>
       <c r="F22" t="b">
         <v>1</v>
@@ -918,13 +918,13 @@
         <v>23</v>
       </c>
       <c r="C23" t="n">
-        <v>21</v>
+        <v>5</v>
       </c>
       <c r="D23" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="E23" t="n">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="F23" t="b">
         <v>0</v>
@@ -964,7 +964,7 @@
         <v>0</v>
       </c>
       <c r="E25" t="n">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="F25" t="b">
         <v>1</v>
@@ -984,7 +984,7 @@
         <v>0</v>
       </c>
       <c r="E26" t="n">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="F26" t="b">
         <v>0</v>
@@ -1004,7 +1004,7 @@
         <v>0</v>
       </c>
       <c r="E27" t="n">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="F27" t="b">
         <v>1</v>
@@ -1044,7 +1044,7 @@
         <v>0</v>
       </c>
       <c r="E29" t="n">
-        <v>82</v>
+        <v>80</v>
       </c>
       <c r="F29" t="b">
         <v>0</v>
@@ -1064,7 +1064,7 @@
         <v>0</v>
       </c>
       <c r="E30" t="n">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="F30" t="b">
         <v>1</v>
@@ -1084,7 +1084,7 @@
         <v>0</v>
       </c>
       <c r="E31" t="n">
-        <v>80</v>
+        <v>75</v>
       </c>
       <c r="F31" t="b">
         <v>1</v>
@@ -1098,13 +1098,13 @@
         <v>24</v>
       </c>
       <c r="C32" t="n">
-        <v>9</v>
+        <v>2</v>
       </c>
       <c r="D32" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
       <c r="E32" t="n">
-        <v>71</v>
+        <v>57</v>
       </c>
       <c r="F32" t="b">
         <v>0</v>
@@ -1124,7 +1124,7 @@
         <v>0</v>
       </c>
       <c r="E33" t="n">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="F33" t="b">
         <v>1</v>
@@ -1164,7 +1164,7 @@
         <v>0</v>
       </c>
       <c r="E35" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="F35" t="b">
         <v>0</v>
@@ -1184,7 +1184,7 @@
         <v>0</v>
       </c>
       <c r="E36" t="n">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="F36" t="b">
         <v>1</v>
@@ -1224,7 +1224,7 @@
         <v>0</v>
       </c>
       <c r="E38" t="n">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="F38" t="b">
         <v>0</v>
@@ -1244,7 +1244,7 @@
         <v>0</v>
       </c>
       <c r="E39" t="n">
-        <v>197</v>
+        <v>184</v>
       </c>
       <c r="F39" t="b">
         <v>1</v>
@@ -1264,7 +1264,7 @@
         <v>0</v>
       </c>
       <c r="E40" t="n">
-        <v>227</v>
+        <v>233</v>
       </c>
       <c r="F40" t="b">
         <v>1</v>
@@ -1278,10 +1278,10 @@
         <v>25</v>
       </c>
       <c r="C41" t="n">
-        <v>14</v>
+        <v>3</v>
       </c>
       <c r="D41" t="n">
-        <v>8</v>
+        <v>3</v>
       </c>
       <c r="E41" t="n">
         <v>204</v>
@@ -1304,7 +1304,7 @@
         <v>0</v>
       </c>
       <c r="E42" t="n">
-        <v>123</v>
+        <v>132</v>
       </c>
       <c r="F42" t="b">
         <v>1</v>
@@ -1324,7 +1324,7 @@
         <v>0</v>
       </c>
       <c r="E43" t="n">
-        <v>91</v>
+        <v>97</v>
       </c>
       <c r="F43" t="b">
         <v>1</v>
@@ -1338,13 +1338,13 @@
         <v>25</v>
       </c>
       <c r="C44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D44" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E44" t="n">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="F44" t="b">
         <v>0</v>
@@ -1364,7 +1364,7 @@
         <v>0</v>
       </c>
       <c r="E45" t="n">
-        <v>136</v>
+        <v>142</v>
       </c>
       <c r="F45" t="b">
         <v>1</v>
@@ -1384,7 +1384,7 @@
         <v>0</v>
       </c>
       <c r="E46" t="n">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="F46" t="b">
         <v>0</v>
@@ -1420,7 +1420,7 @@
         <v>28</v>
       </c>
       <c r="C2" t="n">
-        <v>0.99998789792876</v>
+        <v>0.999988927902842</v>
       </c>
     </row>
     <row r="3">
@@ -1431,7 +1431,7 @@
         <v>29</v>
       </c>
       <c r="C3" t="n">
-        <v>0.984982660004638</v>
+        <v>0.984517272681281</v>
       </c>
     </row>
     <row r="4">
@@ -1442,7 +1442,7 @@
         <v>30</v>
       </c>
       <c r="C4" t="n">
-        <v>0.919210023187344</v>
+        <v>0.915510462152496</v>
       </c>
     </row>
     <row r="5">
@@ -1453,7 +1453,7 @@
         <v>28</v>
       </c>
       <c r="C5" t="n">
-        <v>0.999931777683049</v>
+        <v>0.999922977370381</v>
       </c>
     </row>
     <row r="6">
@@ -1464,7 +1464,7 @@
         <v>29</v>
       </c>
       <c r="C6" t="n">
-        <v>0.939408933471279</v>
+        <v>0.928292177183416</v>
       </c>
     </row>
     <row r="7">
@@ -1475,7 +1475,7 @@
         <v>30</v>
       </c>
       <c r="C7" t="n">
-        <v>0.862872458707852</v>
+        <v>0.860690971710315</v>
       </c>
     </row>
     <row r="8">
@@ -1486,7 +1486,7 @@
         <v>28</v>
       </c>
       <c r="C8" t="n">
-        <v>0.999972913018302</v>
+        <v>0.999971694597877</v>
       </c>
     </row>
     <row r="9">
@@ -1497,7 +1497,7 @@
         <v>29</v>
       </c>
       <c r="C9" t="n">
-        <v>0.973581978807691</v>
+        <v>0.967920670551752</v>
       </c>
     </row>
     <row r="10">
@@ -1508,7 +1508,7 @@
         <v>30</v>
       </c>
       <c r="C10" t="n">
-        <v>0.577520510628317</v>
+        <v>0.572633827877473</v>
       </c>
     </row>
     <row r="11">
@@ -1519,7 +1519,7 @@
         <v>28</v>
       </c>
       <c r="C11" t="n">
-        <v>0.999935831218398</v>
+        <v>0.999922902049992</v>
       </c>
     </row>
     <row r="12">
@@ -1530,7 +1530,7 @@
         <v>29</v>
       </c>
       <c r="C12" t="n">
-        <v>0.343124640524274</v>
+        <v>0.342272874585693</v>
       </c>
     </row>
     <row r="13">
@@ -1541,7 +1541,7 @@
         <v>30</v>
       </c>
       <c r="C13" t="n">
-        <v>0.218701775211784</v>
+        <v>0.192377911156438</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
remove blood by protein identity instead of a threshold nobody could reproduce
</commit_message>
<xml_diff>
--- a/02_Normalization/imputation/c_data/imputation_qc_source_data.xlsx
+++ b/02_Normalization/imputation/c_data/imputation_qc_source_data.xlsx
@@ -498,13 +498,13 @@
         <v>13</v>
       </c>
       <c r="C2" t="n">
-        <v>41</v>
+        <v>43</v>
       </c>
       <c r="D2" t="n">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="E2" t="n">
-        <v>117</v>
+        <v>123</v>
       </c>
       <c r="F2" t="b">
         <v>0</v>
@@ -518,10 +518,10 @@
         <v>13</v>
       </c>
       <c r="C3" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="D3" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E3" t="n">
         <v>77</v>
@@ -538,13 +538,13 @@
         <v>13</v>
       </c>
       <c r="C4" t="n">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="D4" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="E4" t="n">
-        <v>117</v>
+        <v>128</v>
       </c>
       <c r="F4" t="b">
         <v>1</v>
@@ -558,13 +558,13 @@
         <v>13</v>
       </c>
       <c r="C5" t="n">
-        <v>38</v>
+        <v>47</v>
       </c>
       <c r="D5" t="n">
-        <v>27</v>
+        <v>31</v>
       </c>
       <c r="E5" t="n">
-        <v>90</v>
+        <v>107</v>
       </c>
       <c r="F5" t="b">
         <v>0</v>
@@ -578,13 +578,13 @@
         <v>13</v>
       </c>
       <c r="C6" t="n">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="D6" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="E6" t="n">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="F6" t="b">
         <v>1</v>
@@ -598,13 +598,13 @@
         <v>13</v>
       </c>
       <c r="C7" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="D7" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="E7" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F7" t="b">
         <v>1</v>
@@ -618,13 +618,13 @@
         <v>13</v>
       </c>
       <c r="C8" t="n">
-        <v>47</v>
+        <v>51</v>
       </c>
       <c r="D8" t="n">
-        <v>38</v>
+        <v>31</v>
       </c>
       <c r="E8" t="n">
-        <v>119</v>
+        <v>111</v>
       </c>
       <c r="F8" t="b">
         <v>0</v>
@@ -638,13 +638,13 @@
         <v>13</v>
       </c>
       <c r="C9" t="n">
-        <v>27</v>
+        <v>24</v>
       </c>
       <c r="D9" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="E9" t="n">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="F9" t="b">
         <v>1</v>
@@ -658,13 +658,13 @@
         <v>13</v>
       </c>
       <c r="C10" t="n">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="D10" t="n">
-        <v>21</v>
+        <v>17</v>
       </c>
       <c r="E10" t="n">
-        <v>52</v>
+        <v>57</v>
       </c>
       <c r="F10" t="b">
         <v>0</v>
@@ -684,7 +684,7 @@
         <v>0</v>
       </c>
       <c r="E11" t="n">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="F11" t="b">
         <v>0</v>
@@ -704,7 +704,7 @@
         <v>0</v>
       </c>
       <c r="E12" t="n">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F12" t="b">
         <v>1</v>
@@ -724,7 +724,7 @@
         <v>0</v>
       </c>
       <c r="E13" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="F13" t="b">
         <v>1</v>
@@ -741,10 +741,10 @@
         <v>2</v>
       </c>
       <c r="D14" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E14" t="n">
-        <v>40</v>
+        <v>51</v>
       </c>
       <c r="F14" t="b">
         <v>0</v>
@@ -784,7 +784,7 @@
         <v>0</v>
       </c>
       <c r="E16" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F16" t="b">
         <v>1</v>
@@ -804,7 +804,7 @@
         <v>0</v>
       </c>
       <c r="E17" t="n">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="F17" t="b">
         <v>0</v>
@@ -824,7 +824,7 @@
         <v>0</v>
       </c>
       <c r="E18" t="n">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="F18" t="b">
         <v>1</v>
@@ -864,7 +864,7 @@
         <v>0</v>
       </c>
       <c r="E20" t="n">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F20" t="b">
         <v>0</v>
@@ -884,7 +884,7 @@
         <v>0</v>
       </c>
       <c r="E21" t="n">
-        <v>49</v>
+        <v>52</v>
       </c>
       <c r="F21" t="b">
         <v>1</v>
@@ -904,7 +904,7 @@
         <v>0</v>
       </c>
       <c r="E22" t="n">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="F22" t="b">
         <v>1</v>
@@ -918,13 +918,13 @@
         <v>23</v>
       </c>
       <c r="C23" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="D23" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E23" t="n">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="F23" t="b">
         <v>0</v>
@@ -964,7 +964,7 @@
         <v>0</v>
       </c>
       <c r="E25" t="n">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="F25" t="b">
         <v>1</v>
@@ -984,7 +984,7 @@
         <v>0</v>
       </c>
       <c r="E26" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="F26" t="b">
         <v>0</v>
@@ -1004,7 +1004,7 @@
         <v>0</v>
       </c>
       <c r="E27" t="n">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="F27" t="b">
         <v>1</v>
@@ -1024,7 +1024,7 @@
         <v>0</v>
       </c>
       <c r="E28" t="n">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F28" t="b">
         <v>0</v>
@@ -1044,7 +1044,7 @@
         <v>0</v>
       </c>
       <c r="E29" t="n">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="F29" t="b">
         <v>0</v>
@@ -1064,7 +1064,7 @@
         <v>0</v>
       </c>
       <c r="E30" t="n">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="F30" t="b">
         <v>1</v>
@@ -1084,7 +1084,7 @@
         <v>0</v>
       </c>
       <c r="E31" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="F31" t="b">
         <v>1</v>
@@ -1098,13 +1098,13 @@
         <v>24</v>
       </c>
       <c r="C32" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D32" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E32" t="n">
-        <v>57</v>
+        <v>66</v>
       </c>
       <c r="F32" t="b">
         <v>0</v>
@@ -1124,7 +1124,7 @@
         <v>0</v>
       </c>
       <c r="E33" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="F33" t="b">
         <v>1</v>
@@ -1164,7 +1164,7 @@
         <v>0</v>
       </c>
       <c r="E35" t="n">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="F35" t="b">
         <v>0</v>
@@ -1184,7 +1184,7 @@
         <v>0</v>
       </c>
       <c r="E36" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="F36" t="b">
         <v>1</v>
@@ -1224,7 +1224,7 @@
         <v>0</v>
       </c>
       <c r="E38" t="n">
-        <v>195</v>
+        <v>197</v>
       </c>
       <c r="F38" t="b">
         <v>0</v>
@@ -1244,7 +1244,7 @@
         <v>0</v>
       </c>
       <c r="E39" t="n">
-        <v>184</v>
+        <v>189</v>
       </c>
       <c r="F39" t="b">
         <v>1</v>
@@ -1264,7 +1264,7 @@
         <v>0</v>
       </c>
       <c r="E40" t="n">
-        <v>233</v>
+        <v>216</v>
       </c>
       <c r="F40" t="b">
         <v>1</v>
@@ -1278,13 +1278,13 @@
         <v>25</v>
       </c>
       <c r="C41" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="D41" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E41" t="n">
-        <v>204</v>
+        <v>208</v>
       </c>
       <c r="F41" t="b">
         <v>0</v>
@@ -1304,7 +1304,7 @@
         <v>0</v>
       </c>
       <c r="E42" t="n">
-        <v>132</v>
+        <v>118</v>
       </c>
       <c r="F42" t="b">
         <v>1</v>
@@ -1324,7 +1324,7 @@
         <v>0</v>
       </c>
       <c r="E43" t="n">
-        <v>97</v>
+        <v>86</v>
       </c>
       <c r="F43" t="b">
         <v>1</v>
@@ -1338,13 +1338,13 @@
         <v>25</v>
       </c>
       <c r="C44" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="D44" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E44" t="n">
-        <v>175</v>
+        <v>180</v>
       </c>
       <c r="F44" t="b">
         <v>0</v>
@@ -1364,7 +1364,7 @@
         <v>0</v>
       </c>
       <c r="E45" t="n">
-        <v>142</v>
+        <v>138</v>
       </c>
       <c r="F45" t="b">
         <v>1</v>
@@ -1384,7 +1384,7 @@
         <v>0</v>
       </c>
       <c r="E46" t="n">
-        <v>107</v>
+        <v>110</v>
       </c>
       <c r="F46" t="b">
         <v>0</v>
@@ -1420,7 +1420,7 @@
         <v>28</v>
       </c>
       <c r="C2" t="n">
-        <v>0.999988927902842</v>
+        <v>0.999987597799308</v>
       </c>
     </row>
     <row r="3">
@@ -1431,7 +1431,7 @@
         <v>29</v>
       </c>
       <c r="C3" t="n">
-        <v>0.984517272681281</v>
+        <v>0.984036460937735</v>
       </c>
     </row>
     <row r="4">
@@ -1442,7 +1442,7 @@
         <v>30</v>
       </c>
       <c r="C4" t="n">
-        <v>0.915510462152496</v>
+        <v>0.917902902766025</v>
       </c>
     </row>
     <row r="5">
@@ -1453,7 +1453,7 @@
         <v>28</v>
       </c>
       <c r="C5" t="n">
-        <v>0.999922977370381</v>
+        <v>0.999918701641269</v>
       </c>
     </row>
     <row r="6">
@@ -1464,7 +1464,7 @@
         <v>29</v>
       </c>
       <c r="C6" t="n">
-        <v>0.928292177183416</v>
+        <v>0.921003077570767</v>
       </c>
     </row>
     <row r="7">
@@ -1475,7 +1475,7 @@
         <v>30</v>
       </c>
       <c r="C7" t="n">
-        <v>0.860690971710315</v>
+        <v>0.858535007828533</v>
       </c>
     </row>
     <row r="8">
@@ -1486,7 +1486,7 @@
         <v>28</v>
       </c>
       <c r="C8" t="n">
-        <v>0.999971694597877</v>
+        <v>0.999972161966793</v>
       </c>
     </row>
     <row r="9">
@@ -1497,7 +1497,7 @@
         <v>29</v>
       </c>
       <c r="C9" t="n">
-        <v>0.967920670551752</v>
+        <v>0.973589927124417</v>
       </c>
     </row>
     <row r="10">
@@ -1508,7 +1508,7 @@
         <v>30</v>
       </c>
       <c r="C10" t="n">
-        <v>0.572633827877473</v>
+        <v>0.575346706173712</v>
       </c>
     </row>
     <row r="11">
@@ -1519,7 +1519,7 @@
         <v>28</v>
       </c>
       <c r="C11" t="n">
-        <v>0.999922902049992</v>
+        <v>0.999935773255651</v>
       </c>
     </row>
     <row r="12">
@@ -1530,7 +1530,7 @@
         <v>29</v>
       </c>
       <c r="C12" t="n">
-        <v>0.342272874585693</v>
+        <v>0.327791726151665</v>
       </c>
     </row>
     <row r="13">
@@ -1541,7 +1541,7 @@
         <v>30</v>
       </c>
       <c r="C13" t="n">
-        <v>0.192377911156438</v>
+        <v>0.239160026858996</v>
       </c>
     </row>
   </sheetData>

</xml_diff>